<commit_message>
Update screening workbook and agent prompts to latest runs
Replace diffusion_attacks_screening.xlsx and prompts.md with the updated
versions covering the latest screening runs: the catalog grows from 50 to
58 papers (families 4+6+8+18+12+10), the screening log from 154 to 158
records, and the agreement check drops the "post-hoc / supplementary"
framing.

Also refresh README.md to match: updated counts, corrected workbook path,
removal of the stale standalone-catalog and Elsevier class-file notes, and
the citation venue changed to ACM Computing Surveys.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KqSeGseSyFoQjdKzvGDg7Y
</commit_message>
<xml_diff>
--- a/diffusion_attacks_screening.xlsx
+++ b/diffusion_attacks_screening.xlsx
@@ -622,7 +622,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Title/Abstract Screening + Post-Hoc LLM-Agent Agreement</t>
+          <t>Title/Abstract Screening + LLM-Agent Agreement</t>
         </is>
       </c>
     </row>
@@ -682,11 +682,11 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Full-text INCLUDE (final catalog)</t>
+          <t>Final catalog</t>
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -758,7 +758,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="19">
@@ -788,7 +788,7 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Post-hoc LLM-agent agreement check</t>
+          <t>LLM-agent agreement check</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="32">
@@ -984,7 +984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I155"/>
+  <dimension ref="A1:I159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6093,17 +6093,13 @@
       </c>
       <c r="G123" s="6" t="inlineStr">
         <is>
-          <t>EXCLUDE</t>
-        </is>
-      </c>
-      <c r="H123" s="7" t="inlineStr">
-        <is>
-          <t>Found late; not in original catalog. Candidate for follow-up addition.</t>
-        </is>
-      </c>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H123" s="7" t="inlineStr"/>
       <c r="I123" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -6138,17 +6134,13 @@
       </c>
       <c r="G124" s="6" t="inlineStr">
         <is>
-          <t>EXCLUDE</t>
-        </is>
-      </c>
-      <c r="H124" s="7" t="inlineStr">
-        <is>
-          <t>Similar mechanism to IDEATOR; not added to keep catalog manageable.</t>
-        </is>
-      </c>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H124" s="7" t="inlineStr"/>
       <c r="I124" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -6408,17 +6400,13 @@
       </c>
       <c r="G130" s="6" t="inlineStr">
         <is>
-          <t>EXCLUDE</t>
-        </is>
-      </c>
-      <c r="H130" s="7" t="inlineStr">
-        <is>
-          <t>dLLM evaluation; adjacent to DIJA/PAD.</t>
-        </is>
-      </c>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H130" s="7" t="inlineStr"/>
       <c r="I130" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -6633,17 +6621,13 @@
       </c>
       <c r="G135" s="6" t="inlineStr">
         <is>
-          <t>EXCLUDE</t>
-        </is>
-      </c>
-      <c r="H135" s="7" t="inlineStr">
-        <is>
-          <t>Adjacent to CoDefend; could be added in revision.</t>
-        </is>
-      </c>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H135" s="7" t="inlineStr"/>
       <c r="I135" s="6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -7516,6 +7500,170 @@
       <c r="I155" s="6" t="inlineStr">
         <is>
           <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="7" t="inlineStr">
+        <is>
+          <t>2604.08557</t>
+        </is>
+      </c>
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>Re-Mask and Redirect: Exploiting Denoising Irreversibility in Diffusion Language Models</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="inlineStr">
+        <is>
+          <t>Trajectory-level attack on diffusion LLMs: re-masks committed refusal tokens and injects an affirmative prefix (no gradient).</t>
+        </is>
+      </c>
+      <c r="E156" s="7" t="inlineStr">
+        <is>
+          <t>supp</t>
+        </is>
+      </c>
+      <c r="F156" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G156" s="6" t="inlineStr">
+        <is>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H156" s="7" t="inlineStr"/>
+      <c r="I156" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="7" t="inlineStr">
+        <is>
+          <t>openreview:ks5lAv8QDn</t>
+        </is>
+      </c>
+      <c r="C157" s="7" t="inlineStr">
+        <is>
+          <t>DiffTextPure: Defending Large Language Models with Diffusion Purifiers</t>
+        </is>
+      </c>
+      <c r="D157" s="7" t="inlineStr">
+        <is>
+          <t>Plug-and-play diffusion purification of adversarial input text as a pre-processing defense for LLMs.</t>
+        </is>
+      </c>
+      <c r="E157" s="7" t="inlineStr">
+        <is>
+          <t>supp</t>
+        </is>
+      </c>
+      <c r="F157" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G157" s="6" t="inlineStr">
+        <is>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H157" s="7" t="inlineStr"/>
+      <c r="I157" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="6" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="7" t="inlineStr">
+        <is>
+          <t>2410.20971</t>
+        </is>
+      </c>
+      <c r="C158" s="7" t="inlineStr">
+        <is>
+          <t>BlueSuffix: Reinforced Blue Teaming for Vision-Language Models Against Jailbreak Attacks</t>
+        </is>
+      </c>
+      <c r="D158" s="7" t="inlineStr">
+        <is>
+          <t>Bimodal defense: DiffPure image purifier + LLM text purifier + RL-trained blue-team suffix generator.</t>
+        </is>
+      </c>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>supp</t>
+        </is>
+      </c>
+      <c r="F158" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G158" s="6" t="inlineStr">
+        <is>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H158" s="7" t="inlineStr"/>
+      <c r="I158" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="7" t="inlineStr">
+        <is>
+          <t>2504.01308</t>
+        </is>
+      </c>
+      <c r="C159" s="7" t="inlineStr">
+        <is>
+          <t>Safeguarding Vision-Language Models: Mitigating Vulnerabilities to Gaussian Noise in Perturbation-based Attacks</t>
+        </is>
+      </c>
+      <c r="D159" s="7" t="inlineStr">
+        <is>
+          <t>Small-timestep DiffPure purification feeding a Gaussian-noise-tolerant, safety-tuned VLM.</t>
+        </is>
+      </c>
+      <c r="E159" s="7" t="inlineStr">
+        <is>
+          <t>supp</t>
+        </is>
+      </c>
+      <c r="F159" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G159" s="6" t="inlineStr">
+        <is>
+          <t>INCLUDE</t>
+        </is>
+      </c>
+      <c r="H159" s="7" t="inlineStr"/>
+      <c r="I159" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -7531,7 +7679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11520,7 +11668,7 @@
       </c>
       <c r="N51" s="3" t="inlineStr">
         <is>
-          <t>Not released as of the May 2026 cutoff</t>
+          <t>Not released as of the June 2026 cutoff</t>
         </is>
       </c>
       <c r="O51" s="3" t="inlineStr">
@@ -11531,6 +11679,630 @@
       <c r="P51" s="3" t="inlineStr">
         <is>
           <t>Black-box-friendly is useful but joint image+prompt design implies an effective adaptive attack must perturb both modalities; no public code at submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>RedDiffuser: Auditing Multimodal Safety Failures in Vision-Language Models via Reinforced Diffusion</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Wang, Ma</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>arXiv 2025</t>
+        </is>
+      </c>
+      <c r="F52" s="29" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2503.06223</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>E. VLM jailbreak (diffusion as content source)</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Generator (RL-fine-tuned diffusion)</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Latent diffusion (Stable Diffusion); RL-fine-tuned generator for black-box safety auditing</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>RL fine-tuning of the diffusion generator with toxicity + coherence rewards; greedy prompt search</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Multimodal safety-audit prompt set (partial toxic text + visual context)</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>Unsafe-response rate, transferability</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>LLaVA; transfer to Gemini, LLaMA-Vision</t>
+        </is>
+      </c>
+      <c r="N52" s="3" t="inlineStr">
+        <is>
+          <t>Code promised in paper ("we will release"); repo not confirmed live at verification</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="inlineStr">
+        <is>
+          <t>Reinforcement-based framework using diffusion to generate visual contexts for black-box VLM safety auditing; up to +10.69% unsafe-response rate on LLaVA (+8.91% hold-out); transfers to Gemini and LLaMA-Vision; persists under external guardrails</t>
+        </is>
+      </c>
+      <c r="P52" s="3" t="inlineStr">
+        <is>
+          <t>Code only promised (not yet released); scope limited to toxic-continuation auditing rather than general jailbreak; requires RL fine-tuning of the generator.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>VERA-V: Variational Inference Framework for Jailbreaking Vision-Language Models</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Liao, Lochab, Zhang</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>arXiv 2025</t>
+        </is>
+      </c>
+      <c r="F53" s="29" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2510.17759</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>E. Diffusion vs VLM</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>Generator (diffusion synthesis in variational attacker)</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Diffusion image synthesis embedded in a variational-inference attacker over multimodal inputs</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Variational inference; joint text+image adversarial optimization</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Multimodal red-teaming benchmarks</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>ASR, transferability</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>VLMs (open + commercial)</t>
+        </is>
+      </c>
+      <c r="N53" s="3" t="inlineStr">
+        <is>
+          <t>Not confirmed at verification</t>
+        </is>
+      </c>
+      <c r="O53" s="3" t="inlineStr">
+        <is>
+          <t>Variational-inference framework for VLM jailbreak; folds diffusion image synthesis into the attacker; broadens the exposed vulnerability surface vs template attacks</t>
+        </is>
+      </c>
+      <c r="P53" s="3" t="inlineStr">
+        <is>
+          <t>Variational optimization adds attacker-side cost; closed-model transfer and query budget not clearly characterized in the preprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Diffusion-based Cumulative Adversarial Purification for Vision-Language Models</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Fu, Wu, Chen, Peng, Zhang, Cevher, Pashami, Holst</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>TMLR 2026</t>
+        </is>
+      </c>
+      <c r="F54" s="29" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2506.03933</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>C. Defense (multimodal)</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Defense (purification)</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative diffusion purification; Gaussian-noise injection + reverse diffusion on adversarial images</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Training-free cumulative purification</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>VLM adversarial benchmarks</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>ASR, robust accuracy</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>VLMs (captioning / VQA)</t>
+        </is>
+      </c>
+      <c r="N54" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/JasonFu1998/DiffCAP</t>
+        </is>
+      </c>
+      <c r="O54" s="3" t="inlineStr">
+        <is>
+          <t>Cumulative adversarial purification for VLMs; reports its own white-box BPDA+EOT audit of the purifier</t>
+        </is>
+      </c>
+      <c r="P54" s="3" t="inlineStr">
+        <is>
+          <t>Iterative test-time purification adds latency; adaptive robustness is self-audited (BPDA+EOT) rather than independently stress-tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>DiffTextPure: Defending Large Language Models with Diffusion Purifiers</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Anonymous (OpenReview submission)</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>OpenReview submission (anonymized; venue not stated in PDF)</t>
+        </is>
+      </c>
+      <c r="F55" s="29" t="inlineStr">
+        <is>
+          <t>https://openreview.net/forum?id=ks5lAv8QDn</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>C. Defense (text)</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Defense (text purification)</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Discrete-diffusion purification of text (Uniform-perturbation or Absorbing-mask forward process); reverse via concrete-score ancestral sampling</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Training-free; discrete-diffusion purifier as an input pre-processor (no LLM fine-tuning)</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>AdvBench (50 harmful-behaviors subset)</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>Robustness score (defense success %) vs GCG / I-GCG / AutoDAN / ICA attacks</t>
+        </is>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>Llama, Vicuna</t>
+        </is>
+      </c>
+      <c r="N55" s="3" t="inlineStr">
+        <is>
+          <t>Not confirmed at verification</t>
+        </is>
+      </c>
+      <c r="O55" s="3" t="inlineStr">
+        <is>
+          <t>Plug-and-play discrete-diffusion text purifier that generalizes DiffPure to text; pre-processing only, no LLM fine-tuning; Uniform variant reaches ~98% robustness vs GCG, 90-100% vs I-GCG, 94-100% vs AutoDAN on Llama/Vicuna</t>
+        </is>
+      </c>
+      <c r="P55" s="3" t="inlineStr">
+        <is>
+          <t>Unreviewed anonymous preprint; evaluated on a 50-prompt AdvBench subset and older open models (Llama/Vicuna); benign-utility cost and latency not fully characterized.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>BlueSuffix: Reinforced Blue Teaming for Vision-Language Models Against Jailbreak Attacks</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Zhao, Zheng, Luo, Li, Ma, Jiang</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>ICLR 2025</t>
+        </is>
+      </c>
+      <c r="F56" s="29" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2410.20971</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>C. Defense (multimodal)</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Defense (diffusion purification + prompt purifier + suffix generator)</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>Bimodal: DiffPure image purifier + LLM text purifier + RL-trained blue-team suffix generator</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>RL fine-tuning of the suffix generator to maximize an LLM-judge safety score</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>MM-SafetyBench</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>ASR, benign pass rate (BPR), toxicity (Perspective API)</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>LLaVA, MiniGPT-4, InstructBLIP, Gemini</t>
+        </is>
+      </c>
+      <c r="N56" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/Vinsonzyh/BlueSuffix</t>
+        </is>
+      </c>
+      <c r="O56" s="3" t="inlineStr">
+        <is>
+          <t>Bimodal (image+text) defense; reduces ASR by &gt;40% across attack scenarios; BPR ~78% (minimal benign impact)</t>
+        </is>
+      </c>
+      <c r="P56" s="3" t="inlineStr">
+        <is>
+          <t>Three-stage pipeline adds inference cost and requires training the suffix generator; reduces but does not eliminate ASR; evaluated mainly on MM-SafetyBench.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Safeguarding Vision-Language Models: Mitigating Vulnerabilities to Gaussian Noise in Perturbation-based Attacks (DiffPure-VLM)</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Wang, Zuo, Chai, Liu, Fu, Feng, Lam</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>ICCV 2025</t>
+        </is>
+      </c>
+      <c r="F57" s="29" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2504.01308</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>C. Defense (multimodal)</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Defense (purification)</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>DiffPure converts optimization-based adversarial perturbations into Gaussian-like noise handled by a noise-augmented VLM; small-timestep purification (&lt;150 diffusion steps)</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Noise-augmented fine-tuning on the Robust-VLGuard dataset + small-timestep DiffPure image purification</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>RealToxicityPrompts (1,200-prompt challenging subset); MM-Vet (helpfulness); Robust-VLGuard (proposed)</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>ASR (toxicity score &gt; 0.5 via Perspective API / Detoxify); MM-Vet score</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>MiniGPT-4, LLaVA-1.5, InternVL2, LLaMA-3.2-Vision-11B, Qwen2.5-VL-7B, Ivy-VLM-3B</t>
+        </is>
+      </c>
+      <c r="N57" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/JarvisUSTC/DiffPure-RobustVLM</t>
+        </is>
+      </c>
+      <c r="O57" s="3" t="inlineStr">
+        <is>
+          <t>Two-part defense: Robust-VLGuard (noise-augmented multimodal safety dataset + fine-tuning) and DiffPure-VLM, which uses diffusion to convert optimization-based perturbations into Gaussian-like noise the hardened VLM tolerates; brings ASR to near-clean levels within &lt;150 diffusion steps while preserving MM-Vet helpfulness; outperforms JailGuard preprocessing</t>
+        </is>
+      </c>
+      <c r="P57" s="3" t="inlineStr">
+        <is>
+          <t>Requires noise-augmented fine-tuning of the VLM (not plug-and-play) and adds diffusion latency; targets optimization-based perturbations more than semantic/typographic attacks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Re-Mask and Redirect: Exploiting Denoising Irreversibility in Diffusion Language Models</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Singh</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>arXiv 2026</t>
+        </is>
+      </c>
+      <c r="F58" s="29" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2604.08557</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>B. dLLM safety (victim = dLLM)</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Target (dLLM is the victim model)</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Trajectory-level attack: re-masks committed refusal tokens + injects an affirmative prefix; no gradient</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Training-free trajectory manipulation (re-mask + redirect)</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>HarmBench</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>ASR</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>Three publicly available safety-tuned dLLMs (incl. the A2D defense)</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
+        <is>
+          <t>Not publicly released (no code in paper)</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr">
+        <is>
+          <t>First trajectory-level attack on dLLMs; 74-82% ASR on HarmBench, 92-98% with a generic 8-token prefix; both components necessary; gradient optimization degrades ASR; 'Defense Inversion Effect' makes the A2D defense MORE vulnerable (89.9%) than undefended</t>
+        </is>
+      </c>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>Single-author preprint with no released code; requires white-box access to the intermediate denoising trajectory; evaluated only on three open dLLMs, closed-model applicability untested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Safer by Diffusion, Broken by Context: Diffusion LLM's Safety Blessing and Its Failure Mode</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>He, Chen, Lin, Wang, Chang, Sommerlade, Torr, Yu, Bibi, Yu</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>arXiv 2026</t>
+        </is>
+      </c>
+      <c r="F59" s="29" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2602.00388</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>B. dLLM safety (victim = dLLM)</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Target (dLLM is the victim model)</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Empirical safety analysis of dLLMs + context-nesting jailbreak</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Empirical study + context-nesting attack</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>JailbreakBench, HarmBench</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>ASR-K, ASR-E, harmfulness score (GPT-judge)</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>LLaDA, Dream, Gemini Diffusion</t>
+        </is>
+      </c>
+      <c r="N59" s="3" t="inlineStr">
+        <is>
+          <t>Not confirmed at verification</t>
+        </is>
+      </c>
+      <c r="O59" s="3" t="inlineStr">
+        <is>
+          <t>dLLMs are safer against input jailbreaks via a 'stepwise reduction effect' (GCG 16% vs ~50% on AR-LLMs) but broken by context nesting; reports the first jailbreak of Gemini Diffusion</t>
+        </is>
+      </c>
+      <c r="P59" s="3" t="inlineStr">
+        <is>
+          <t>Primarily an empirical safety characterization; the context-nesting jailbreak is demonstrated but not broadly benchmarked against strong baselines; code not confirmed released.</t>
         </is>
       </c>
     </row>
@@ -11566,7 +12338,7 @@
     <row r="2">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t>Compiled May 2026 for Abrar's LLM-red-teaming-via-diffusion project.</t>
+          <t>Compiled June 2026 for Abrar's LLM-red-teaming-via-diffusion project.</t>
         </is>
       </c>
     </row>
@@ -13776,6 +14548,80 @@
         <v>6</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="22" t="n">
+        <v>57</v>
+      </c>
+      <c r="B52" s="23" t="inlineStr">
+        <is>
+          <t>Re-Mask and Redirect / TRAJHIJACK (Singh, 2026)</t>
+        </is>
+      </c>
+      <c r="C52" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G52" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I52" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J52" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="22" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="n">
+        <v>58</v>
+      </c>
+      <c r="B53" s="23" t="inlineStr">
+        <is>
+          <t>Safer by Diffusion (He et al., 2026)</t>
+        </is>
+      </c>
+      <c r="C53" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I53" s="22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J53" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="22" t="n">
+        <v>6</v>
+      </c>
+    </row>
     <row r="54">
       <c r="B54" s="10" t="inlineStr">
         <is>

</xml_diff>